<commit_message>
Add course-to-month mapping and Trend Index to LIV leaderboard
- Filter and sort courses by month order
- Add Trend Index (current avg vs previous avg)
- Fix LIV Total calculation for active courses only
</commit_message>
<xml_diff>
--- a/data/GOAM_Scores_2026_May_updated.xlsx
+++ b/data/GOAM_Scores_2026_May_updated.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>CopperLeaf</t>
+          <t>PGC</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -454,11 +454,6 @@
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>PGC</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
         <is>
           <t>Rounds_Played</t>
         </is>
@@ -480,15 +475,12 @@
         <v>36</v>
       </c>
       <c r="E2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F2" t="n">
         <v>37</v>
       </c>
       <c r="G2" t="n">
-        <v>32</v>
-      </c>
-      <c r="H2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -508,15 +500,12 @@
         <v>35</v>
       </c>
       <c r="E3" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F3" t="n">
         <v>35</v>
       </c>
       <c r="G3" t="n">
-        <v>32</v>
-      </c>
-      <c r="H3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -536,15 +525,12 @@
         <v>33</v>
       </c>
       <c r="E4" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="F4" t="n">
         <v>29</v>
       </c>
       <c r="G4" t="n">
-        <v>35</v>
-      </c>
-      <c r="H4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -564,15 +550,12 @@
         <v>35</v>
       </c>
       <c r="E5" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F5" t="n">
         <v>27</v>
       </c>
       <c r="G5" t="n">
-        <v>31</v>
-      </c>
-      <c r="H5" t="n">
         <v>4</v>
       </c>
     </row>
@@ -592,15 +575,12 @@
         <v>33</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F6" t="n">
         <v>36</v>
       </c>
       <c r="G6" t="n">
-        <v>26</v>
-      </c>
-      <c r="H6" t="n">
         <v>3</v>
       </c>
     </row>
@@ -620,15 +600,12 @@
         <v>25</v>
       </c>
       <c r="E7" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F7" t="n">
         <v>29</v>
       </c>
       <c r="G7" t="n">
-        <v>22</v>
-      </c>
-      <c r="H7" t="n">
         <v>4</v>
       </c>
     </row>
@@ -648,15 +625,12 @@
         <v>40</v>
       </c>
       <c r="E8" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>30</v>
-      </c>
-      <c r="H8" t="n">
         <v>3</v>
       </c>
     </row>
@@ -676,15 +650,12 @@
         <v>32</v>
       </c>
       <c r="E9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>27</v>
-      </c>
-      <c r="H9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -704,15 +675,12 @@
         <v>35</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F10" t="n">
         <v>24</v>
       </c>
       <c r="G10" t="n">
-        <v>23</v>
-      </c>
-      <c r="H10" t="n">
         <v>3</v>
       </c>
     </row>
@@ -732,15 +700,12 @@
         <v>29</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F11" t="n">
         <v>25</v>
       </c>
       <c r="G11" t="n">
-        <v>28</v>
-      </c>
-      <c r="H11" t="n">
         <v>3</v>
       </c>
     </row>
@@ -760,15 +725,12 @@
         <v>30</v>
       </c>
       <c r="E12" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>27</v>
-      </c>
-      <c r="H12" t="n">
         <v>3</v>
       </c>
     </row>
@@ -788,15 +750,12 @@
         <v>28</v>
       </c>
       <c r="E13" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
         <v>28</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
         <v>3</v>
       </c>
     </row>
@@ -816,15 +775,12 @@
         <v>36</v>
       </c>
       <c r="E14" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -844,15 +800,12 @@
         <v>19</v>
       </c>
       <c r="E15" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>29</v>
-      </c>
-      <c r="H15" t="n">
         <v>3</v>
       </c>
     </row>
@@ -872,15 +825,12 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F16" t="n">
         <v>37</v>
       </c>
       <c r="G16" t="n">
-        <v>35</v>
-      </c>
-      <c r="H16" t="n">
         <v>2</v>
       </c>
     </row>
@@ -900,15 +850,12 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F17" t="n">
         <v>34</v>
       </c>
       <c r="G17" t="n">
-        <v>35</v>
-      </c>
-      <c r="H17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -928,15 +875,12 @@
         <v>36</v>
       </c>
       <c r="E18" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -956,15 +900,12 @@
         <v>14</v>
       </c>
       <c r="E19" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>22</v>
-      </c>
-      <c r="H19" t="n">
         <v>3</v>
       </c>
     </row>
@@ -984,15 +925,12 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>31</v>
-      </c>
-      <c r="H20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1018,9 +956,6 @@
         <v>31</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1040,15 +975,12 @@
         <v>31</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>20</v>
-      </c>
-      <c r="H22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1068,15 +1000,12 @@
         <v>15</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>30</v>
-      </c>
-      <c r="H23" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1102,9 +1031,6 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1124,15 +1050,12 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1158,9 +1081,6 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1186,9 +1106,6 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1208,15 +1125,12 @@
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>23</v>
-      </c>
-      <c r="H28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1231,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1257,7 +1171,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>CopperLeaf</t>
+          <t>PGC</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -1266,11 +1180,6 @@
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>PGC</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
         <is>
           <t>Games_Played</t>
         </is>
@@ -1292,15 +1201,12 @@
         <v>16</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F2" t="n">
         <v>11</v>
       </c>
       <c r="G2" t="n">
-        <v>15</v>
-      </c>
-      <c r="H2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1320,15 +1226,12 @@
         <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
         <v>18</v>
       </c>
       <c r="G3" t="n">
-        <v>9</v>
-      </c>
-      <c r="H3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1348,15 +1251,12 @@
         <v>17</v>
       </c>
       <c r="E4" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
         <v>27</v>
       </c>
       <c r="G4" t="n">
-        <v>19</v>
-      </c>
-      <c r="H4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1376,15 +1276,12 @@
         <v>24</v>
       </c>
       <c r="E5" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F5" t="n">
         <v>23</v>
       </c>
       <c r="G5" t="n">
-        <v>24</v>
-      </c>
-      <c r="H5" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1404,15 +1301,12 @@
         <v>26</v>
       </c>
       <c r="E6" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F6" t="n">
         <v>21</v>
       </c>
       <c r="G6" t="n">
-        <v>28</v>
-      </c>
-      <c r="H6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1432,15 +1326,12 @@
         <v>19</v>
       </c>
       <c r="E7" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1466,9 +1357,6 @@
         <v>22</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1488,15 +1376,12 @@
         <v>20</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F9" t="n">
         <v>22</v>
       </c>
       <c r="G9" t="n">
-        <v>22</v>
-      </c>
-      <c r="H9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1516,15 +1401,12 @@
         <v>20</v>
       </c>
       <c r="E10" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>23</v>
-      </c>
-      <c r="H10" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1544,15 +1426,12 @@
         <v>27</v>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>21</v>
-      </c>
-      <c r="H11" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1572,15 +1451,12 @@
         <v>24</v>
       </c>
       <c r="E12" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
         <v>23</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1600,15 +1476,12 @@
         <v>25</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F13" t="n">
         <v>21</v>
       </c>
       <c r="G13" t="n">
-        <v>29</v>
-      </c>
-      <c r="H13" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1628,15 +1501,12 @@
         <v>18</v>
       </c>
       <c r="E14" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>23</v>
-      </c>
-      <c r="H14" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1656,15 +1526,12 @@
         <v>21</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F15" t="n">
         <v>32</v>
       </c>
       <c r="G15" t="n">
-        <v>30</v>
-      </c>
-      <c r="H15" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1684,15 +1551,12 @@
         <v>30</v>
       </c>
       <c r="E16" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>28</v>
-      </c>
-      <c r="H16" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1712,15 +1576,12 @@
         <v>40</v>
       </c>
       <c r="E17" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>43</v>
-      </c>
-      <c r="H17" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1740,15 +1601,12 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>10</v>
-      </c>
-      <c r="H18" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1774,9 +1632,6 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1796,15 +1651,12 @@
         <v>14</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1830,9 +1682,6 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1852,15 +1701,12 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F22" t="n">
         <v>18</v>
       </c>
       <c r="G22" t="n">
-        <v>15</v>
-      </c>
-      <c r="H22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1880,15 +1726,12 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F23" t="n">
         <v>21</v>
       </c>
       <c r="G23" t="n">
-        <v>18</v>
-      </c>
-      <c r="H23" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1908,15 +1751,12 @@
         <v>27</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>36</v>
-      </c>
-      <c r="H24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1936,15 +1776,12 @@
         <v>40</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>34</v>
-      </c>
-      <c r="H25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1964,15 +1801,12 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1992,15 +1826,12 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>31</v>
-      </c>
-      <c r="H27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2026,9 +1857,6 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2043,7 +1871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2074,17 +1902,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>CopperLeaf</t>
+          <t>PGC</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
           <t>Kyalami</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>PGC</t>
         </is>
       </c>
     </row>
@@ -2109,14 +1932,11 @@
         <v>108</v>
       </c>
       <c r="F2" t="n">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="G2" t="n">
         <v>103</v>
       </c>
-      <c r="H2" t="n">
-        <v>102</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2139,14 +1959,11 @@
         <v>104</v>
       </c>
       <c r="F3" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="G3" t="n">
         <v>63</v>
       </c>
-      <c r="H3" t="n">
-        <v>86</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2169,14 +1986,11 @@
         <v>102</v>
       </c>
       <c r="F4" t="n">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="G4" t="n">
         <v>53</v>
       </c>
-      <c r="H4" t="n">
-        <v>76</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2199,14 +2013,11 @@
         <v>102</v>
       </c>
       <c r="F5" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G5" t="n">
         <v>37</v>
       </c>
-      <c r="H5" t="n">
-        <v>86</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2229,13 +2040,10 @@
         <v>57</v>
       </c>
       <c r="F6" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="G6" t="n">
         <v>87</v>
-      </c>
-      <c r="H6" t="n">
-        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix course filtering and display in leaderboards
- Show only active courses (month <= current) in filter dropdown
- Exclude Services and invalid sheets
- Default to active courses for leaderboard display
</commit_message>
<xml_diff>
--- a/data/GOAM_Scores_2026_May_updated.xlsx
+++ b/data/GOAM_Scores_2026_May_updated.xlsx
@@ -1892,7 +1892,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>Trend Index</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -1918,14 +1918,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>389</v>
+        <v>313</v>
       </c>
       <c r="C2" t="n">
-        <v>97.2</v>
+        <v>104.3</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1945,10 +1945,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>334</v>
+        <v>253</v>
       </c>
       <c r="C3" t="n">
-        <v>83.5</v>
+        <v>84.3</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1968,41 +1968,41 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tee Tigers</t>
+          <t>Birdie Buddies</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>333</v>
+        <v>238</v>
       </c>
       <c r="C4" t="n">
-        <v>83.2</v>
+        <v>79.3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>102</v>
+        <v>57</v>
       </c>
       <c r="F4" t="n">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="G4" t="n">
-        <v>53</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Home Boys</t>
+          <t>Tee Tigers</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>309</v>
+        <v>231</v>
       </c>
       <c r="C5" t="n">
-        <v>77.2</v>
+        <v>77</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2013,23 +2013,23 @@
         <v>102</v>
       </c>
       <c r="F5" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="G5" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Birdie Buddies</t>
+          <t>Home Boys</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>294</v>
+        <v>225</v>
       </c>
       <c r="C6" t="n">
-        <v>73.5</v>
+        <v>75</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -2037,13 +2037,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="F6" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="G6" t="n">
-        <v>87</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Ranking for IPS
</commit_message>
<xml_diff>
--- a/data/GOAM_Scores_2026_May_updated.xlsx
+++ b/data/GOAM_Scores_2026_May_updated.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strokes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LIV" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Akasia" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kyalami" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PGC" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CopperLeaf" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kyalami" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PGC" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +455,11 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>CopperLeaf</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Rounds_Played</t>
         </is>
       </c>
@@ -468,7 +474,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>105</v>
+        <v>139</v>
       </c>
       <c r="D2" t="n">
         <v>36</v>
@@ -480,7 +486,10 @@
         <v>37</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>34</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -493,7 +502,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="D3" t="n">
         <v>35</v>
@@ -505,7 +514,10 @@
         <v>35</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>30</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -518,7 +530,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>97</v>
+        <v>125</v>
       </c>
       <c r="D4" t="n">
         <v>33</v>
@@ -530,7 +542,10 @@
         <v>29</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>28</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -539,23 +554,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Warren Lottering</t>
+          <t>Jodi Van Niekerk</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="D5" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E5" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F5" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>24</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -564,22 +582,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Jodi Van Niekerk</t>
+          <t>Warren Lottering</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D6" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E6" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F6" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
         <v>3</v>
       </c>
     </row>
@@ -589,23 +610,26 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ashley Spocter</t>
+          <t>Ranzel Louw</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E7" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>16</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -614,22 +638,25 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Byron Labuschagne</t>
+          <t>Trevor Meyer</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D8" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="E8" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F8" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
+        <v>18</v>
+      </c>
+      <c r="H8" t="n">
         <v>3</v>
       </c>
     </row>
@@ -639,22 +666,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ranzel Louw</t>
+          <t>Dale Adonis</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E9" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F9" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
+        <v>26</v>
+      </c>
+      <c r="H9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -664,23 +694,26 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chad Naude</t>
+          <t>Ashley Spocter</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="E10" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="F10" t="n">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -689,23 +722,26 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Trevor Meyer</t>
+          <t>Byron Labuschagne</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="E11" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -714,23 +750,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bjorn Singh</t>
+          <t>Eugene Dudley</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E12" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="F12" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>24</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -739,23 +778,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dale Adonis</t>
+          <t>Shaheen Boughan</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="D13" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E13" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>24</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -764,22 +806,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Eugene Dudley</t>
+          <t>John Barker</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D14" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E14" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
+        <v>38</v>
+      </c>
+      <c r="H14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -789,23 +834,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Shaheen Boughan</t>
+          <t>Laurent Changuion</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="D15" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F15" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>25</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -814,23 +862,26 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dewald Van Rooyen</t>
+          <t>Chad Naude</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="D16" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F16" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="G16" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -839,22 +890,25 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Godfrey Daniels</t>
+          <t>Bjorn Singh</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="D17" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -864,23 +918,26 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Laurent Changuion</t>
+          <t>Winston Willemse</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="D18" t="n">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="E18" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>2</v>
+        <v>32</v>
+      </c>
+      <c r="H18" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -889,23 +946,26 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Lenny Booysen</t>
+          <t>Pieter Gagiano</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="D19" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E19" t="n">
+        <v>22</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
         <v>30</v>
       </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>2</v>
+      <c r="H19" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -914,22 +974,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pieter Gagiano</t>
+          <t>Shawn Davies</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="D20" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
+        <v>32</v>
+      </c>
+      <c r="H20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -939,23 +1002,26 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Winston Willemse</t>
+          <t>Dewald Van Rooyen</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="D21" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -964,23 +1030,26 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>John Barker</t>
+          <t>Godfrey Daniels</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="D22" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -989,22 +1058,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fuad Adams</t>
+          <t>Lenny Booysen</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D23" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1014,23 +1086,26 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Shawn Davies</t>
+          <t>Fuad Adams</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="E24" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -1039,14 +1114,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Arn Smith</t>
+          <t>Ronny Kaptein</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D25" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -1055,7 +1130,10 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>34</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1064,14 +1142,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Brian Plaatjies</t>
+          <t>Arn Smith</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D26" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -1080,7 +1158,10 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -1089,22 +1170,53 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>Brian Plaatjies</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>24</v>
+      </c>
+      <c r="D27" t="n">
+        <v>24</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Kirsten Jacobs</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="C28" t="n">
         <v>23</v>
       </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
         <v>23</v>
       </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="n">
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1119,7 +1231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1155,6 +1267,11 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>CopperLeaf</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Games_Played</t>
         </is>
       </c>
@@ -1169,7 +1286,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="D2" t="n">
         <v>16</v>
@@ -1181,7 +1298,10 @@
         <v>11</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>13</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1194,7 +1314,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D3" t="n">
         <v>15</v>
@@ -1206,7 +1326,10 @@
         <v>18</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -1215,23 +1338,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dewald Van Rooyen</t>
+          <t>Jodi Van Niekerk</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="D4" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>28</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -1240,23 +1366,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jodi Van Niekerk</t>
+          <t>Lucien Barnes</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>63</v>
+        <v>98</v>
       </c>
       <c r="D5" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="E5" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F5" t="n">
+        <v>23</v>
+      </c>
+      <c r="G5" t="n">
         <v>27</v>
       </c>
-      <c r="G5" t="n">
-        <v>3</v>
+      <c r="H5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -1265,23 +1394,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Byron Labuschagne</t>
+          <t>Ranzel Louw</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E6" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>30</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1290,22 +1422,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lucien Barnes</t>
+          <t>Winston Willemse</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E7" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
+        <v>22</v>
+      </c>
+      <c r="H7" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1315,22 +1450,25 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ranzel Louw</t>
+          <t>Dewald Van Rooyen</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="D8" t="n">
         <v>26</v>
       </c>
       <c r="E8" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1340,22 +1478,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Warren Lottering</t>
+          <t>Byron Labuschagne</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E9" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1365,22 +1506,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ashley Spocter</t>
+          <t>Dale Adonis</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="D10" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" t="n">
+        <v>23</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
         <v>21</v>
       </c>
-      <c r="E10" t="n">
-        <v>30</v>
-      </c>
-      <c r="F10" t="n">
-        <v>32</v>
-      </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1390,23 +1534,26 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Winston Willemse</t>
+          <t>Laurent Changuion</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19</v>
+        <v>66</v>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>18</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -1415,23 +1562,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fuad Adams</t>
+          <t>Shaheen Boughan</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="D12" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>24</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1440,23 +1590,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arn Smith</t>
+          <t>Warren Lottering</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="D13" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1465,23 +1618,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Chad Naude</t>
+          <t>Trevor Meyer</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E14" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F14" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>38</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1490,23 +1646,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bjorn Singh</t>
+          <t>Ashley Spocter</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>39</v>
+        <v>83</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E15" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F15" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1515,23 +1674,26 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Trevor Meyer</t>
+          <t>Eugene Dudley</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>41</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="E16" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>32</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1540,23 +1702,26 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dale Adonis</t>
+          <t>Pieter Gagiano</t>
         </is>
       </c>
       <c r="C17" t="n">
+        <v>123</v>
+      </c>
+      <c r="D17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" t="n">
         <v>43</v>
       </c>
-      <c r="D17" t="n">
-        <v>20</v>
-      </c>
-      <c r="E17" t="n">
-        <v>23</v>
-      </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>2</v>
+        <v>40</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -1565,22 +1730,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shaheen Boughan</t>
+          <t>Shawn Davies</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D18" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1590,22 +1758,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Laurent Changuion</t>
+          <t>Fuad Adams</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="D19" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E19" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1615,22 +1786,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Eugene Dudley</t>
+          <t>John Barker</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="D20" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E20" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
+        <v>8</v>
+      </c>
+      <c r="H20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1640,22 +1814,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Godfrey Daniels</t>
+          <t>Arn Smith</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="D21" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E21" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1665,22 +1842,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Lenny Booysen</t>
+          <t>Chad Naude</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="D22" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1690,22 +1870,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pieter Gagiano</t>
+          <t>Bjorn Singh</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="D23" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1715,23 +1898,26 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Shawn Davies</t>
+          <t>Godfrey Daniels</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E24" t="n">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -1740,23 +1926,26 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>John Barker</t>
+          <t>Lenny Booysen</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="D25" t="n">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -1765,22 +1954,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kirsten Jacobs</t>
+          <t>Ronny Kaptein</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
       </c>
       <c r="G26" t="n">
+        <v>16</v>
+      </c>
+      <c r="H26" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1790,22 +1982,53 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>Kirsten Jacobs</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>31</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>31</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Brian Plaatjies</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="C28" t="n">
         <v>33</v>
       </c>
-      <c r="D27" t="n">
+      <c r="D28" t="n">
         <v>33</v>
       </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="n">
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1820,7 +2043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1859,6 +2082,11 @@
           <t>Kyalami</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CopperLeaf</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1867,10 +2095,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>313</v>
+        <v>389</v>
       </c>
       <c r="C2" t="n">
-        <v>104.3</v>
+        <v>97.2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1886,6 +2114,9 @@
       <c r="G2" t="n">
         <v>103</v>
       </c>
+      <c r="H2" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1894,10 +2125,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>253</v>
+        <v>334</v>
       </c>
       <c r="C3" t="n">
-        <v>84.3</v>
+        <v>83.5</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1913,18 +2144,21 @@
       <c r="G3" t="n">
         <v>63</v>
       </c>
+      <c r="H3" t="n">
+        <v>81</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Birdie Buddies</t>
+          <t>Tee Tigers</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>238</v>
+        <v>333</v>
       </c>
       <c r="C4" t="n">
-        <v>79.3</v>
+        <v>83.2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1932,53 +2166,59 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="F4" t="n">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="G4" t="n">
-        <v>87</v>
+        <v>53</v>
+      </c>
+      <c r="H4" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tee Tigers</t>
+          <t>Home Boys</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>231</v>
+        <v>309</v>
       </c>
       <c r="C5" t="n">
-        <v>77</v>
+        <v>77.2</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>102</v>
       </c>
       <c r="F5" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G5" t="n">
-        <v>53</v>
+        <v>37</v>
+      </c>
+      <c r="H5" t="n">
+        <v>84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Home Boys</t>
+          <t>Birdie Buddies</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>225</v>
+        <v>294</v>
       </c>
       <c r="C6" t="n">
-        <v>75</v>
+        <v>73.5</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1986,13 +2226,16 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>102</v>
+        <v>57</v>
       </c>
       <c r="F6" t="n">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G6" t="n">
-        <v>37</v>
+        <v>87</v>
+      </c>
+      <c r="H6" t="n">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2444,7 +2687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2472,18 +2715,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Chad Naude</t>
+          <t>John Barker</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Fairway Fighters</t>
+          <t>Tee Tigers</t>
         </is>
       </c>
     </row>
@@ -2494,10 +2737,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C3" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2508,68 +2751,68 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Warren Lottering</t>
+          <t>Ronny Kaptein</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C4" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tee Stingers</t>
+          <t>Tee Tigers</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lucien Barnes</t>
+          <t>Shawn Davies</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="C5" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fairway Fighters</t>
+          <t>Birdie Buddies</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bjorn Singh</t>
+          <t>Winston Willemse</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C6" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Birdie Buddies</t>
+          <t>Tee Stingers</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dewald Van Rooyen</t>
+          <t>Lucien Barnes</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C7" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -2580,68 +2823,68 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mika Moerat</t>
+          <t>Pieter Gagiano</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>90</v>
+        <v>112</v>
       </c>
       <c r="C8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Fairway Fighters</t>
+          <t>Tee Tigers</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ranzel Louw</t>
+          <t>Mika Moerat</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tee Tigers</t>
+          <t>Fairway Fighters</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Shaheen Boughan</t>
+          <t>Dale Adonis</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C10" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Birdie Buddies</t>
+          <t>Home Boys</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jodi Van Niekerk</t>
+          <t>Laurent Changuion</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="C11" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2652,14 +2895,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Byron Labuschagne</t>
+          <t>Shaheen Boughan</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C12" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2670,7 +2913,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ashley Spocter</t>
+          <t>Eugene Dudley</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2680,6 +2923,60 @@
         <v>24</v>
       </c>
       <c r="D13" t="inlineStr">
+        <is>
+          <t>Home Boys</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Jodi Van Niekerk</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>100</v>
+      </c>
+      <c r="C14" t="n">
+        <v>24</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Tee Stingers</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Trevor Meyer</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>110</v>
+      </c>
+      <c r="C15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Fairway Fighters</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ranzel Louw</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>102</v>
+      </c>
+      <c r="C16" t="n">
+        <v>16</v>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>Tee Tigers</t>
         </is>
@@ -2696,6 +2993,258 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Strokes</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>IPS</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Chad Naude</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>90</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Fairway Fighters</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Arno Adonis</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>83</v>
+      </c>
+      <c r="C3" t="n">
+        <v>37</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Home Boys</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Warren Lottering</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>93</v>
+      </c>
+      <c r="C4" t="n">
+        <v>36</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tee Stingers</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lucien Barnes</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>95</v>
+      </c>
+      <c r="C5" t="n">
+        <v>35</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fairway Fighters</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bjorn Singh</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>93</v>
+      </c>
+      <c r="C6" t="n">
+        <v>34</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Birdie Buddies</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Dewald Van Rooyen</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>94</v>
+      </c>
+      <c r="C7" t="n">
+        <v>31</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Fairway Fighters</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mika Moerat</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>90</v>
+      </c>
+      <c r="C8" t="n">
+        <v>29</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Fairway Fighters</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ranzel Louw</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>93</v>
+      </c>
+      <c r="C9" t="n">
+        <v>29</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Tee Tigers</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Shaheen Boughan</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>95</v>
+      </c>
+      <c r="C10" t="n">
+        <v>28</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Birdie Buddies</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jodi Van Niekerk</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>99</v>
+      </c>
+      <c r="C11" t="n">
+        <v>27</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Tee Stingers</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Byron Labuschagne</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>94</v>
+      </c>
+      <c r="C12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Birdie Buddies</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ashley Spocter</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>104</v>
+      </c>
+      <c r="C13" t="n">
+        <v>24</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Tee Tigers</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Plenty of stuff - User logon was a nightmare
</commit_message>
<xml_diff>
--- a/data/GOAM_Scores_2026_May_updated.xlsx
+++ b/data/GOAM_Scores_2026_May_updated.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,35 +430,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Pos Change</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Best6_IPS</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Akasia</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>PGC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Kyalami</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>CopperLeaf</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Rounds_Played</t>
         </is>
@@ -470,25 +475,30 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Arno Adonis</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>139</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>36</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>32</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>37</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>34</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -498,25 +508,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Lucien Barnes</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>132</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>35</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>32</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>35</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>30</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -526,25 +541,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Mika Moerat</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>125</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>33</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>35</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>29</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>28</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -554,25 +574,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Jodi Van Niekerk</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>117</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>35</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>31</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>27</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>24</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>4</v>
       </c>
     </row>
@@ -582,25 +607,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Warren Lottering</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>95</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>33</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>26</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>36</v>
       </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
       <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
         <v>3</v>
       </c>
     </row>
@@ -610,25 +640,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>Ranzel Louw</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>92</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>25</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>22</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>29</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>16</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>4</v>
       </c>
     </row>
@@ -638,25 +673,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Trevor Meyer</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>88</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>40</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>30</v>
       </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
       <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>18</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>3</v>
       </c>
     </row>
@@ -666,25 +706,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Dale Adonis</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>85</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>32</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>27</v>
       </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
       <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>26</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -694,25 +739,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Ashley Spocter</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>82</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>35</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>23</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>24</v>
       </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
       <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
         <v>3</v>
       </c>
     </row>
@@ -722,25 +772,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>Byron Labuschagne</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>82</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>29</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>28</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>25</v>
       </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
       <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
         <v>3</v>
       </c>
     </row>
@@ -750,25 +805,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>Eugene Dudley</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>81</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>30</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>27</v>
       </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
       <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
         <v>24</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>3</v>
       </c>
     </row>
@@ -778,25 +838,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>Shaheen Boughan</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>80</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>28</v>
       </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
       <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
         <v>28</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>24</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>3</v>
       </c>
     </row>
@@ -806,25 +871,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>John Barker</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>74</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>36</v>
       </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
         <v>38</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -834,25 +904,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>Laurent Changuion</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="D15" t="n">
         <v>73</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>19</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>29</v>
       </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
       <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
         <v>25</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>3</v>
       </c>
     </row>
@@ -862,25 +937,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>Chad Naude</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>72</v>
       </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
       <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
         <v>35</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>37</v>
       </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
       <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
         <v>2</v>
       </c>
     </row>
@@ -890,25 +970,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>Bjorn Singh</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="D17" t="n">
         <v>69</v>
       </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
       <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
         <v>35</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>34</v>
       </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
       <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -918,25 +1003,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>Winston Willemse</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>68</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>36</v>
       </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
         <v>32</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -946,25 +1036,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>Pieter Gagiano</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>66</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>14</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>22</v>
       </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
       <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
         <v>30</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>3</v>
       </c>
     </row>
@@ -974,25 +1069,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Shawn Davies</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="D20" t="n">
         <v>63</v>
       </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
       <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
         <v>31</v>
       </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
       <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
         <v>32</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1002,25 +1102,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>Dewald Van Rooyen</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="n">
         <v>55</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>24</v>
       </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
       <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
         <v>31</v>
       </c>
-      <c r="G21" t="n">
-        <v>0</v>
-      </c>
       <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1030,25 +1135,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>Godfrey Daniels</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="D22" t="n">
         <v>51</v>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>31</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>20</v>
       </c>
-      <c r="F22" t="n">
-        <v>0</v>
-      </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1058,25 +1168,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>Lenny Booysen</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="D23" t="n">
         <v>45</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>15</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>30</v>
       </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1086,17 +1201,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>Fuad Adams</t>
         </is>
-      </c>
-      <c r="C24" t="n">
-        <v>34</v>
       </c>
       <c r="D24" t="n">
         <v>34</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1105,6 +1222,9 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1114,15 +1234,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Ronny Kaptein</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="D25" t="n">
         <v>34</v>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
@@ -1130,9 +1252,12 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
         <v>34</v>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1142,17 +1267,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>Arn Smith</t>
         </is>
-      </c>
-      <c r="C26" t="n">
-        <v>28</v>
       </c>
       <c r="D26" t="n">
         <v>28</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1161,6 +1288,9 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1170,17 +1300,19 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>Brian Plaatjies</t>
         </is>
-      </c>
-      <c r="C27" t="n">
-        <v>24</v>
       </c>
       <c r="D27" t="n">
         <v>24</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1189,6 +1321,9 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1198,25 +1333,30 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>Kirsten Jacobs</t>
         </is>
       </c>
-      <c r="C28" t="n">
+      <c r="D28" t="n">
         <v>23</v>
       </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
       <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
         <v>23</v>
       </c>
-      <c r="F28" t="n">
-        <v>0</v>
-      </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
       <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>